<commit_message>
Add staff attendance, searchable student pickers and editable student gender
</commit_message>
<xml_diff>
--- a/public/KCC-Student-Upload-Template.xlsx
+++ b/public/KCC-Student-Upload-Template.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" r:id="R477fa380211847c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="1" r:id="R0a935a4220984b11"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -292,6 +292,7 @@
     <x:col min="1" max="1" width="8" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="65" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="44" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -304,6 +305,9 @@
       <x:c r="C1" s="5" t="str">
         <x:v>SCHOOL</x:v>
       </x:c>
+      <x:c r="D1" s="5" t="str">
+        <x:v>GENDER</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
       <x:c r="A2" s="6" t="n">
@@ -311,6 +315,7 @@
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
+      <x:c r="D2" s="8"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="6" t="n">
@@ -318,6 +323,7 @@
       </x:c>
       <x:c r="B3" s="8"/>
       <x:c r="C3" s="8"/>
+      <x:c r="D3" s="8"/>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="6" t="n">
@@ -325,6 +331,7 @@
       </x:c>
       <x:c r="B4" s="8"/>
       <x:c r="C4" s="8"/>
+      <x:c r="D4" s="8"/>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="6" t="n">
@@ -332,6 +339,7 @@
       </x:c>
       <x:c r="B5" s="8"/>
       <x:c r="C5" s="8"/>
+      <x:c r="D5" s="8"/>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="6" t="n">
@@ -339,6 +347,7 @@
       </x:c>
       <x:c r="B6" s="8"/>
       <x:c r="C6" s="8"/>
+      <x:c r="D6" s="8"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="6" t="n">
@@ -346,6 +355,7 @@
       </x:c>
       <x:c r="B7" s="8"/>
       <x:c r="C7" s="8"/>
+      <x:c r="D7" s="8"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="6" t="n">
@@ -353,6 +363,7 @@
       </x:c>
       <x:c r="B8" s="8"/>
       <x:c r="C8" s="8"/>
+      <x:c r="D8" s="8"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="6" t="n">
@@ -360,6 +371,7 @@
       </x:c>
       <x:c r="B9" s="8"/>
       <x:c r="C9" s="8"/>
+      <x:c r="D9" s="8"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="6" t="n">
@@ -367,6 +379,7 @@
       </x:c>
       <x:c r="B10" s="8"/>
       <x:c r="C10" s="8"/>
+      <x:c r="D10" s="8"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="6" t="n">
@@ -374,6 +387,7 @@
       </x:c>
       <x:c r="B11" s="8"/>
       <x:c r="C11" s="8"/>
+      <x:c r="D11" s="8"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="6" t="n">
@@ -381,6 +395,7 @@
       </x:c>
       <x:c r="B12" s="8"/>
       <x:c r="C12" s="8"/>
+      <x:c r="D12" s="8"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="6" t="n">
@@ -388,6 +403,7 @@
       </x:c>
       <x:c r="B13" s="8"/>
       <x:c r="C13" s="8"/>
+      <x:c r="D13" s="8"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="6" t="n">
@@ -395,6 +411,7 @@
       </x:c>
       <x:c r="B14" s="8"/>
       <x:c r="C14" s="8"/>
+      <x:c r="D14" s="8"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="6" t="n">
@@ -402,6 +419,7 @@
       </x:c>
       <x:c r="B15" s="8"/>
       <x:c r="C15" s="8"/>
+      <x:c r="D15" s="8"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="6" t="n">
@@ -409,6 +427,7 @@
       </x:c>
       <x:c r="B16" s="8"/>
       <x:c r="C16" s="8"/>
+      <x:c r="D16" s="8"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="6" t="n">
@@ -416,6 +435,7 @@
       </x:c>
       <x:c r="B17" s="8"/>
       <x:c r="C17" s="8"/>
+      <x:c r="D17" s="8"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="6" t="n">
@@ -423,6 +443,7 @@
       </x:c>
       <x:c r="B18" s="8"/>
       <x:c r="C18" s="8"/>
+      <x:c r="D18" s="8"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="6" t="n">
@@ -430,6 +451,7 @@
       </x:c>
       <x:c r="B19" s="8"/>
       <x:c r="C19" s="8"/>
+      <x:c r="D19" s="8"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="6" t="n">
@@ -437,6 +459,7 @@
       </x:c>
       <x:c r="B20" s="8"/>
       <x:c r="C20" s="8"/>
+      <x:c r="D20" s="8"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="6" t="n">
@@ -444,6 +467,7 @@
       </x:c>
       <x:c r="B21" s="8"/>
       <x:c r="C21" s="8"/>
+      <x:c r="D21" s="8"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="6" t="n">
@@ -451,6 +475,7 @@
       </x:c>
       <x:c r="B22" s="8"/>
       <x:c r="C22" s="8"/>
+      <x:c r="D22" s="8"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="6" t="n">
@@ -458,6 +483,7 @@
       </x:c>
       <x:c r="B23" s="8"/>
       <x:c r="C23" s="8"/>
+      <x:c r="D23" s="8"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="6" t="n">
@@ -465,6 +491,7 @@
       </x:c>
       <x:c r="B24" s="8"/>
       <x:c r="C24" s="8"/>
+      <x:c r="D24" s="8"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="6" t="n">
@@ -472,6 +499,7 @@
       </x:c>
       <x:c r="B25" s="8"/>
       <x:c r="C25" s="8"/>
+      <x:c r="D25" s="8"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="6" t="n">
@@ -479,6 +507,7 @@
       </x:c>
       <x:c r="B26" s="8"/>
       <x:c r="C26" s="8"/>
+      <x:c r="D26" s="8"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="6" t="n">
@@ -486,6 +515,7 @@
       </x:c>
       <x:c r="B27" s="8"/>
       <x:c r="C27" s="8"/>
+      <x:c r="D27" s="8"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="6" t="n">
@@ -493,6 +523,7 @@
       </x:c>
       <x:c r="B28" s="8"/>
       <x:c r="C28" s="8"/>
+      <x:c r="D28" s="8"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="6" t="n">
@@ -500,6 +531,7 @@
       </x:c>
       <x:c r="B29" s="8"/>
       <x:c r="C29" s="8"/>
+      <x:c r="D29" s="8"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="6" t="n">
@@ -507,6 +539,7 @@
       </x:c>
       <x:c r="B30" s="8"/>
       <x:c r="C30" s="8"/>
+      <x:c r="D30" s="8"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="6" t="n">
@@ -514,6 +547,7 @@
       </x:c>
       <x:c r="B31" s="8"/>
       <x:c r="C31" s="8"/>
+      <x:c r="D31" s="8"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="6" t="n">
@@ -521,6 +555,7 @@
       </x:c>
       <x:c r="B32" s="8"/>
       <x:c r="C32" s="8"/>
+      <x:c r="D32" s="8"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="6" t="n">
@@ -528,6 +563,7 @@
       </x:c>
       <x:c r="B33" s="8"/>
       <x:c r="C33" s="8"/>
+      <x:c r="D33" s="8"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="6" t="n">
@@ -535,6 +571,7 @@
       </x:c>
       <x:c r="B34" s="8"/>
       <x:c r="C34" s="8"/>
+      <x:c r="D34" s="8"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="6" t="n">
@@ -542,6 +579,7 @@
       </x:c>
       <x:c r="B35" s="8"/>
       <x:c r="C35" s="8"/>
+      <x:c r="D35" s="8"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="6" t="n">
@@ -549,6 +587,7 @@
       </x:c>
       <x:c r="B36" s="8"/>
       <x:c r="C36" s="8"/>
+      <x:c r="D36" s="8"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="6" t="n">
@@ -556,6 +595,7 @@
       </x:c>
       <x:c r="B37" s="8"/>
       <x:c r="C37" s="8"/>
+      <x:c r="D37" s="8"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="6" t="n">
@@ -563,6 +603,7 @@
       </x:c>
       <x:c r="B38" s="8"/>
       <x:c r="C38" s="8"/>
+      <x:c r="D38" s="8"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="6" t="n">
@@ -570,6 +611,7 @@
       </x:c>
       <x:c r="B39" s="8"/>
       <x:c r="C39" s="8"/>
+      <x:c r="D39" s="8"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="6" t="n">
@@ -577,6 +619,7 @@
       </x:c>
       <x:c r="B40" s="8"/>
       <x:c r="C40" s="8"/>
+      <x:c r="D40" s="8"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="6" t="n">
@@ -584,6 +627,7 @@
       </x:c>
       <x:c r="B41" s="8"/>
       <x:c r="C41" s="8"/>
+      <x:c r="D41" s="8"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="6" t="n">
@@ -591,6 +635,7 @@
       </x:c>
       <x:c r="B42" s="8"/>
       <x:c r="C42" s="8"/>
+      <x:c r="D42" s="8"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="6" t="n">
@@ -598,6 +643,7 @@
       </x:c>
       <x:c r="B43" s="8"/>
       <x:c r="C43" s="8"/>
+      <x:c r="D43" s="8"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="6" t="n">
@@ -605,6 +651,7 @@
       </x:c>
       <x:c r="B44" s="8"/>
       <x:c r="C44" s="8"/>
+      <x:c r="D44" s="8"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="6" t="n">
@@ -612,6 +659,7 @@
       </x:c>
       <x:c r="B45" s="8"/>
       <x:c r="C45" s="8"/>
+      <x:c r="D45" s="8"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="6" t="n">
@@ -619,6 +667,7 @@
       </x:c>
       <x:c r="B46" s="8"/>
       <x:c r="C46" s="8"/>
+      <x:c r="D46" s="8"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="6" t="n">
@@ -626,6 +675,7 @@
       </x:c>
       <x:c r="B47" s="8"/>
       <x:c r="C47" s="8"/>
+      <x:c r="D47" s="8"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="6" t="n">
@@ -633,6 +683,7 @@
       </x:c>
       <x:c r="B48" s="8"/>
       <x:c r="C48" s="8"/>
+      <x:c r="D48" s="8"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="6" t="n">
@@ -640,6 +691,7 @@
       </x:c>
       <x:c r="B49" s="8"/>
       <x:c r="C49" s="8"/>
+      <x:c r="D49" s="8"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="6" t="n">
@@ -647,6 +699,7 @@
       </x:c>
       <x:c r="B50" s="8"/>
       <x:c r="C50" s="8"/>
+      <x:c r="D50" s="8"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="6" t="n">
@@ -654,6 +707,7 @@
       </x:c>
       <x:c r="B51" s="8"/>
       <x:c r="C51" s="8"/>
+      <x:c r="D51" s="8"/>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="6" t="n">
@@ -661,6 +715,7 @@
       </x:c>
       <x:c r="B52" s="8"/>
       <x:c r="C52" s="8"/>
+      <x:c r="D52" s="8"/>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="6" t="n">
@@ -668,6 +723,7 @@
       </x:c>
       <x:c r="B53" s="8"/>
       <x:c r="C53" s="8"/>
+      <x:c r="D53" s="8"/>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="6" t="n">
@@ -675,6 +731,7 @@
       </x:c>
       <x:c r="B54" s="8"/>
       <x:c r="C54" s="8"/>
+      <x:c r="D54" s="8"/>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
       <x:c r="A55" s="6" t="n">
@@ -682,6 +739,7 @@
       </x:c>
       <x:c r="B55" s="8"/>
       <x:c r="C55" s="8"/>
+      <x:c r="D55" s="8"/>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="6" t="n">
@@ -689,6 +747,7 @@
       </x:c>
       <x:c r="B56" s="8"/>
       <x:c r="C56" s="8"/>
+      <x:c r="D56" s="8"/>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="6" t="n">
@@ -696,6 +755,7 @@
       </x:c>
       <x:c r="B57" s="8"/>
       <x:c r="C57" s="8"/>
+      <x:c r="D57" s="8"/>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="6" t="n">
@@ -703,6 +763,7 @@
       </x:c>
       <x:c r="B58" s="8"/>
       <x:c r="C58" s="8"/>
+      <x:c r="D58" s="8"/>
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
       <x:c r="A59" s="6" t="n">
@@ -710,6 +771,7 @@
       </x:c>
       <x:c r="B59" s="8"/>
       <x:c r="C59" s="8"/>
+      <x:c r="D59" s="8"/>
     </x:row>
     <x:row r="60" ht="23" customHeight="1">
       <x:c r="A60" s="6" t="n">
@@ -717,6 +779,7 @@
       </x:c>
       <x:c r="B60" s="8"/>
       <x:c r="C60" s="8"/>
+      <x:c r="D60" s="8"/>
     </x:row>
     <x:row r="61" ht="23" customHeight="1">
       <x:c r="A61" s="6" t="n">
@@ -724,6 +787,7 @@
       </x:c>
       <x:c r="B61" s="8"/>
       <x:c r="C61" s="8"/>
+      <x:c r="D61" s="8"/>
     </x:row>
     <x:row r="62" ht="23" customHeight="1">
       <x:c r="A62" s="6" t="n">
@@ -731,6 +795,7 @@
       </x:c>
       <x:c r="B62" s="8"/>
       <x:c r="C62" s="8"/>
+      <x:c r="D62" s="8"/>
     </x:row>
     <x:row r="63" ht="23" customHeight="1">
       <x:c r="A63" s="6" t="n">
@@ -738,6 +803,7 @@
       </x:c>
       <x:c r="B63" s="8"/>
       <x:c r="C63" s="8"/>
+      <x:c r="D63" s="8"/>
     </x:row>
     <x:row r="64" ht="23" customHeight="1">
       <x:c r="A64" s="6" t="n">
@@ -745,6 +811,7 @@
       </x:c>
       <x:c r="B64" s="8"/>
       <x:c r="C64" s="8"/>
+      <x:c r="D64" s="8"/>
     </x:row>
     <x:row r="65" ht="23" customHeight="1">
       <x:c r="A65" s="6" t="n">
@@ -752,6 +819,7 @@
       </x:c>
       <x:c r="B65" s="8"/>
       <x:c r="C65" s="8"/>
+      <x:c r="D65" s="8"/>
     </x:row>
     <x:row r="66" ht="23" customHeight="1">
       <x:c r="A66" s="6" t="n">
@@ -759,6 +827,7 @@
       </x:c>
       <x:c r="B66" s="8"/>
       <x:c r="C66" s="8"/>
+      <x:c r="D66" s="8"/>
     </x:row>
     <x:row r="67" ht="23" customHeight="1">
       <x:c r="A67" s="6" t="n">
@@ -766,6 +835,7 @@
       </x:c>
       <x:c r="B67" s="8"/>
       <x:c r="C67" s="8"/>
+      <x:c r="D67" s="8"/>
     </x:row>
     <x:row r="68" ht="23" customHeight="1">
       <x:c r="A68" s="6" t="n">
@@ -773,6 +843,7 @@
       </x:c>
       <x:c r="B68" s="8"/>
       <x:c r="C68" s="8"/>
+      <x:c r="D68" s="8"/>
     </x:row>
     <x:row r="69" ht="23" customHeight="1">
       <x:c r="A69" s="6" t="n">
@@ -780,6 +851,7 @@
       </x:c>
       <x:c r="B69" s="8"/>
       <x:c r="C69" s="8"/>
+      <x:c r="D69" s="8"/>
     </x:row>
     <x:row r="70" ht="23" customHeight="1">
       <x:c r="A70" s="6" t="n">
@@ -787,6 +859,7 @@
       </x:c>
       <x:c r="B70" s="8"/>
       <x:c r="C70" s="8"/>
+      <x:c r="D70" s="8"/>
     </x:row>
     <x:row r="71" ht="23" customHeight="1">
       <x:c r="A71" s="6" t="n">
@@ -794,6 +867,7 @@
       </x:c>
       <x:c r="B71" s="8"/>
       <x:c r="C71" s="8"/>
+      <x:c r="D71" s="8"/>
     </x:row>
     <x:row r="72" ht="23" customHeight="1">
       <x:c r="A72" s="6" t="n">
@@ -801,6 +875,7 @@
       </x:c>
       <x:c r="B72" s="8"/>
       <x:c r="C72" s="8"/>
+      <x:c r="D72" s="8"/>
     </x:row>
     <x:row r="73" ht="23" customHeight="1">
       <x:c r="A73" s="6" t="n">
@@ -808,6 +883,7 @@
       </x:c>
       <x:c r="B73" s="8"/>
       <x:c r="C73" s="8"/>
+      <x:c r="D73" s="8"/>
     </x:row>
     <x:row r="74" ht="23" customHeight="1">
       <x:c r="A74" s="6" t="n">
@@ -815,6 +891,7 @@
       </x:c>
       <x:c r="B74" s="8"/>
       <x:c r="C74" s="8"/>
+      <x:c r="D74" s="8"/>
     </x:row>
     <x:row r="75" ht="23" customHeight="1">
       <x:c r="A75" s="6" t="n">
@@ -822,6 +899,7 @@
       </x:c>
       <x:c r="B75" s="8"/>
       <x:c r="C75" s="8"/>
+      <x:c r="D75" s="8"/>
     </x:row>
     <x:row r="76" ht="23" customHeight="1">
       <x:c r="A76" s="6" t="n">
@@ -829,6 +907,7 @@
       </x:c>
       <x:c r="B76" s="8"/>
       <x:c r="C76" s="8"/>
+      <x:c r="D76" s="8"/>
     </x:row>
     <x:row r="77" ht="23" customHeight="1">
       <x:c r="A77" s="6" t="n">
@@ -836,6 +915,7 @@
       </x:c>
       <x:c r="B77" s="8"/>
       <x:c r="C77" s="8"/>
+      <x:c r="D77" s="8"/>
     </x:row>
     <x:row r="78" ht="23" customHeight="1">
       <x:c r="A78" s="6" t="n">
@@ -843,6 +923,7 @@
       </x:c>
       <x:c r="B78" s="8"/>
       <x:c r="C78" s="8"/>
+      <x:c r="D78" s="8"/>
     </x:row>
     <x:row r="79" ht="23" customHeight="1">
       <x:c r="A79" s="6" t="n">
@@ -850,6 +931,7 @@
       </x:c>
       <x:c r="B79" s="8"/>
       <x:c r="C79" s="8"/>
+      <x:c r="D79" s="8"/>
     </x:row>
     <x:row r="80" ht="23" customHeight="1">
       <x:c r="A80" s="6" t="n">
@@ -857,6 +939,7 @@
       </x:c>
       <x:c r="B80" s="8"/>
       <x:c r="C80" s="8"/>
+      <x:c r="D80" s="8"/>
     </x:row>
     <x:row r="81" ht="23" customHeight="1">
       <x:c r="A81" s="6" t="n">
@@ -864,6 +947,7 @@
       </x:c>
       <x:c r="B81" s="8"/>
       <x:c r="C81" s="8"/>
+      <x:c r="D81" s="8"/>
     </x:row>
     <x:row r="82" ht="23" customHeight="1">
       <x:c r="A82" s="6" t="n">
@@ -871,6 +955,7 @@
       </x:c>
       <x:c r="B82" s="8"/>
       <x:c r="C82" s="8"/>
+      <x:c r="D82" s="8"/>
     </x:row>
     <x:row r="83" ht="23" customHeight="1">
       <x:c r="A83" s="6" t="n">
@@ -878,6 +963,7 @@
       </x:c>
       <x:c r="B83" s="8"/>
       <x:c r="C83" s="8"/>
+      <x:c r="D83" s="8"/>
     </x:row>
     <x:row r="84" ht="23" customHeight="1">
       <x:c r="A84" s="6" t="n">
@@ -885,6 +971,7 @@
       </x:c>
       <x:c r="B84" s="8"/>
       <x:c r="C84" s="8"/>
+      <x:c r="D84" s="8"/>
     </x:row>
     <x:row r="85" ht="23" customHeight="1">
       <x:c r="A85" s="6" t="n">
@@ -892,6 +979,7 @@
       </x:c>
       <x:c r="B85" s="8"/>
       <x:c r="C85" s="8"/>
+      <x:c r="D85" s="8"/>
     </x:row>
     <x:row r="86" ht="23" customHeight="1">
       <x:c r="A86" s="6" t="n">
@@ -899,6 +987,7 @@
       </x:c>
       <x:c r="B86" s="8"/>
       <x:c r="C86" s="8"/>
+      <x:c r="D86" s="8"/>
     </x:row>
     <x:row r="87" ht="23" customHeight="1">
       <x:c r="A87" s="6" t="n">
@@ -906,6 +995,7 @@
       </x:c>
       <x:c r="B87" s="8"/>
       <x:c r="C87" s="8"/>
+      <x:c r="D87" s="8"/>
     </x:row>
     <x:row r="88" ht="23" customHeight="1">
       <x:c r="A88" s="6" t="n">
@@ -913,6 +1003,7 @@
       </x:c>
       <x:c r="B88" s="8"/>
       <x:c r="C88" s="8"/>
+      <x:c r="D88" s="8"/>
     </x:row>
     <x:row r="89" ht="23" customHeight="1">
       <x:c r="A89" s="6" t="n">
@@ -920,6 +1011,7 @@
       </x:c>
       <x:c r="B89" s="8"/>
       <x:c r="C89" s="8"/>
+      <x:c r="D89" s="8"/>
     </x:row>
     <x:row r="90" ht="23" customHeight="1">
       <x:c r="A90" s="6" t="n">
@@ -927,6 +1019,7 @@
       </x:c>
       <x:c r="B90" s="8"/>
       <x:c r="C90" s="8"/>
+      <x:c r="D90" s="8"/>
     </x:row>
     <x:row r="91" ht="23" customHeight="1">
       <x:c r="A91" s="6" t="n">
@@ -934,6 +1027,7 @@
       </x:c>
       <x:c r="B91" s="8"/>
       <x:c r="C91" s="8"/>
+      <x:c r="D91" s="8"/>
     </x:row>
     <x:row r="92" ht="23" customHeight="1">
       <x:c r="A92" s="6" t="n">
@@ -941,6 +1035,7 @@
       </x:c>
       <x:c r="B92" s="8"/>
       <x:c r="C92" s="8"/>
+      <x:c r="D92" s="8"/>
     </x:row>
     <x:row r="93" ht="23" customHeight="1">
       <x:c r="A93" s="6" t="n">
@@ -948,6 +1043,7 @@
       </x:c>
       <x:c r="B93" s="8"/>
       <x:c r="C93" s="8"/>
+      <x:c r="D93" s="8"/>
     </x:row>
     <x:row r="94" ht="23" customHeight="1">
       <x:c r="A94" s="6" t="n">
@@ -955,6 +1051,7 @@
       </x:c>
       <x:c r="B94" s="8"/>
       <x:c r="C94" s="8"/>
+      <x:c r="D94" s="8"/>
     </x:row>
     <x:row r="95" ht="23" customHeight="1">
       <x:c r="A95" s="6" t="n">
@@ -962,6 +1059,7 @@
       </x:c>
       <x:c r="B95" s="8"/>
       <x:c r="C95" s="8"/>
+      <x:c r="D95" s="8"/>
     </x:row>
     <x:row r="96" ht="23" customHeight="1">
       <x:c r="A96" s="6" t="n">
@@ -969,6 +1067,7 @@
       </x:c>
       <x:c r="B96" s="8"/>
       <x:c r="C96" s="8"/>
+      <x:c r="D96" s="8"/>
     </x:row>
     <x:row r="97" ht="23" customHeight="1">
       <x:c r="A97" s="6" t="n">
@@ -976,6 +1075,7 @@
       </x:c>
       <x:c r="B97" s="8"/>
       <x:c r="C97" s="8"/>
+      <x:c r="D97" s="8"/>
     </x:row>
     <x:row r="98" ht="23" customHeight="1">
       <x:c r="A98" s="6" t="n">
@@ -983,6 +1083,7 @@
       </x:c>
       <x:c r="B98" s="8"/>
       <x:c r="C98" s="8"/>
+      <x:c r="D98" s="8"/>
     </x:row>
     <x:row r="99" ht="23" customHeight="1">
       <x:c r="A99" s="6" t="n">
@@ -990,6 +1091,7 @@
       </x:c>
       <x:c r="B99" s="8"/>
       <x:c r="C99" s="8"/>
+      <x:c r="D99" s="8"/>
     </x:row>
     <x:row r="100" ht="23" customHeight="1">
       <x:c r="A100" s="6" t="n">
@@ -997,6 +1099,7 @@
       </x:c>
       <x:c r="B100" s="8"/>
       <x:c r="C100" s="8"/>
+      <x:c r="D100" s="8"/>
     </x:row>
     <x:row r="101" ht="23" customHeight="1">
       <x:c r="A101" s="6" t="n">
@@ -1004,8 +1107,14 @@
       </x:c>
       <x:c r="B101" s="8"/>
       <x:c r="C101" s="8"/>
+      <x:c r="D101" s="8"/>
     </x:row>
   </x:sheetData>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="D2:D401">
+      <x:formula1>"Male,Female,Not specified"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>